<commit_message>
Update plasmid dynamics analyses and figures
</commit_message>
<xml_diff>
--- a/Keio_Community/indiv_halflife/raw_data/LT23_KeioV3_indiv_plating.xlsx
+++ b/Keio_Community/indiv_halflife/raw_data/LT23_KeioV3_indiv_plating.xlsx
@@ -5,17 +5,19 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johnkingzhou/Library/CloudStorage/Dropbox/Ghost effect/Experimental/LT23 Keio indiv GE/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johnkingzhou/Library/CloudStorage/Dropbox/Ghost effect/Experimental/LT23&amp;24 Keio indiv GE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C30685C-7380-7E42-B088-2938E3FAF926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59A39393-0C55-0C48-ACA5-719F4F8A8E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27580" yWindow="8740" windowWidth="25600" windowHeight="14400" activeTab="2" xr2:uid="{E42DBC6F-C817-EB4F-BD27-70423367A304}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="25600" windowHeight="14280" activeTab="2" xr2:uid="{E42DBC6F-C817-EB4F-BD27-70423367A304}"/>
   </bookViews>
   <sheets>
     <sheet name="Day0" sheetId="1" r:id="rId1"/>
     <sheet name="Day3" sheetId="14" r:id="rId2"/>
     <sheet name="Day6" sheetId="15" r:id="rId3"/>
+    <sheet name="Day9" sheetId="16" r:id="rId4"/>
+    <sheet name="Day14" sheetId="17" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="17">
   <si>
     <t>LB</t>
   </si>
@@ -57,6 +59,39 @@
   </si>
   <si>
     <t>#4+R6K</t>
+  </si>
+  <si>
+    <t>Raw</t>
+  </si>
+  <si>
+    <t>LB: 2e6</t>
+  </si>
+  <si>
+    <t>Plasmid: 2e6</t>
+  </si>
+  <si>
+    <t>LB: 1e6</t>
+  </si>
+  <si>
+    <t>Plasmid: 2e5</t>
+  </si>
+  <si>
+    <t>Dilution rates</t>
+  </si>
+  <si>
+    <t>Plasmid: 1e6</t>
+  </si>
+  <si>
+    <t>Plasmid: 1e5</t>
+  </si>
+  <si>
+    <t>Carb: 1e6</t>
+  </si>
+  <si>
+    <t>Rep1: LB: 1e6; Strp: 1e6</t>
+  </si>
+  <si>
+    <t>Rep2&amp;3: LB: 2e6; Strp: 1e6</t>
   </si>
 </sst>
 </file>
@@ -648,15 +683,15 @@
         <v>100</v>
       </c>
       <c r="G5" s="1">
-        <f>D5*$B$5/100</f>
+        <f t="shared" ref="G5:I7" si="4">D5*$B$5/100</f>
         <v>90</v>
       </c>
       <c r="H5" s="1">
-        <f>E5*$B$5/100</f>
+        <f t="shared" si="4"/>
         <v>90</v>
       </c>
       <c r="I5" s="1">
-        <f>F5*$B$5/100</f>
+        <f t="shared" si="4"/>
         <v>90</v>
       </c>
       <c r="J5" s="2"/>
@@ -697,15 +732,15 @@
         <v>100</v>
       </c>
       <c r="G6" s="1">
-        <f>D6*$B$5/100</f>
+        <f t="shared" si="4"/>
         <v>90</v>
       </c>
       <c r="H6" s="1">
-        <f>E6*$B$5/100</f>
+        <f t="shared" si="4"/>
         <v>90</v>
       </c>
       <c r="I6" s="1">
-        <f>F6*$B$5/100</f>
+        <f t="shared" si="4"/>
         <v>90</v>
       </c>
       <c r="J6" s="2"/>
@@ -744,15 +779,15 @@
         <v>100</v>
       </c>
       <c r="G7" s="1">
-        <f>D7*$B$5/100</f>
+        <f t="shared" si="4"/>
         <v>90</v>
       </c>
       <c r="H7" s="1">
-        <f>E7*$B$5/100</f>
+        <f t="shared" si="4"/>
         <v>90</v>
       </c>
       <c r="I7" s="1">
-        <f>F7*$B$5/100</f>
+        <f t="shared" si="4"/>
         <v>90</v>
       </c>
       <c r="J7" s="2"/>
@@ -793,15 +828,15 @@
         <v>100</v>
       </c>
       <c r="G8" s="1">
-        <f>D8*$B$8/100</f>
+        <f t="shared" ref="G8:I10" si="5">D8*$B$8/100</f>
         <v>50</v>
       </c>
       <c r="H8" s="1">
-        <f>E8*$B$8/100</f>
+        <f t="shared" si="5"/>
         <v>50</v>
       </c>
       <c r="I8" s="1">
-        <f>F8*$B$8/100</f>
+        <f t="shared" si="5"/>
         <v>50</v>
       </c>
       <c r="J8" s="2"/>
@@ -842,15 +877,15 @@
         <v>100</v>
       </c>
       <c r="G9" s="1">
-        <f>D9*$B$8/100</f>
+        <f t="shared" si="5"/>
         <v>50</v>
       </c>
       <c r="H9" s="1">
-        <f>E9*$B$8/100</f>
+        <f t="shared" si="5"/>
         <v>50</v>
       </c>
       <c r="I9" s="1">
-        <f>F9*$B$8/100</f>
+        <f t="shared" si="5"/>
         <v>50</v>
       </c>
       <c r="J9" s="2"/>
@@ -889,15 +924,15 @@
         <v>100</v>
       </c>
       <c r="G10" s="1">
-        <f>D10*$B$8/100</f>
+        <f t="shared" si="5"/>
         <v>50</v>
       </c>
       <c r="H10" s="1">
-        <f>E10*$B$8/100</f>
+        <f t="shared" si="5"/>
         <v>50</v>
       </c>
       <c r="I10" s="1">
-        <f>F10*$B$8/100</f>
+        <f t="shared" si="5"/>
         <v>50</v>
       </c>
       <c r="J10" s="2"/>
@@ -944,11 +979,11 @@
         <v>100</v>
       </c>
       <c r="H11" s="1">
-        <f t="shared" ref="H11:H13" si="4">E11*$B$2/100</f>
+        <f t="shared" ref="H11:H13" si="6">E11*$B$2/100</f>
         <v>100</v>
       </c>
       <c r="I11" s="1">
-        <f t="shared" ref="I11:I13" si="5">F11*$B$2/100</f>
+        <f t="shared" ref="I11:I13" si="7">F11*$B$2/100</f>
         <v>100</v>
       </c>
       <c r="N11" s="1"/>
@@ -988,15 +1023,15 @@
         <v>100</v>
       </c>
       <c r="G12" s="1">
-        <f t="shared" ref="G12:G13" si="6">D12*$B$2/100</f>
+        <f t="shared" ref="G12:G13" si="8">D12*$B$2/100</f>
         <v>100</v>
       </c>
       <c r="H12" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>100</v>
       </c>
       <c r="I12" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>100</v>
       </c>
       <c r="N12" s="1"/>
@@ -1034,15 +1069,15 @@
         <v>100</v>
       </c>
       <c r="G13" s="1">
+        <f t="shared" si="8"/>
+        <v>100</v>
+      </c>
+      <c r="H13" s="1">
         <f t="shared" si="6"/>
         <v>100</v>
       </c>
-      <c r="H13" s="1">
-        <f t="shared" si="4"/>
-        <v>100</v>
-      </c>
       <c r="I13" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>100</v>
       </c>
       <c r="N13" s="1"/>
@@ -1082,15 +1117,15 @@
         <v>100</v>
       </c>
       <c r="G14" s="1">
-        <f>D14*$B$5/100</f>
+        <f t="shared" ref="G14:I16" si="9">D14*$B$5/100</f>
         <v>90</v>
       </c>
       <c r="H14" s="1">
-        <f>E14*$B$5/100</f>
+        <f t="shared" si="9"/>
         <v>90</v>
       </c>
       <c r="I14" s="1">
-        <f>F14*$B$5/100</f>
+        <f t="shared" si="9"/>
         <v>90</v>
       </c>
       <c r="J14" s="2"/>
@@ -1121,15 +1156,15 @@
         <v>100</v>
       </c>
       <c r="G15" s="1">
-        <f>D15*$B$5/100</f>
+        <f t="shared" si="9"/>
         <v>90</v>
       </c>
       <c r="H15" s="1">
-        <f>E15*$B$5/100</f>
+        <f t="shared" si="9"/>
         <v>90</v>
       </c>
       <c r="I15" s="1">
-        <f>F15*$B$5/100</f>
+        <f t="shared" si="9"/>
         <v>90</v>
       </c>
       <c r="J15" s="2"/>
@@ -1158,15 +1193,15 @@
         <v>100</v>
       </c>
       <c r="G16" s="1">
-        <f>D16*$B$5/100</f>
+        <f t="shared" si="9"/>
         <v>90</v>
       </c>
       <c r="H16" s="1">
-        <f>E16*$B$5/100</f>
+        <f t="shared" si="9"/>
         <v>90</v>
       </c>
       <c r="I16" s="1">
-        <f>F16*$B$5/100</f>
+        <f t="shared" si="9"/>
         <v>90</v>
       </c>
       <c r="J16" s="2"/>
@@ -1197,15 +1232,15 @@
         <v>100</v>
       </c>
       <c r="G17" s="1">
-        <f>D17*$B$8/100</f>
+        <f t="shared" ref="G17:I19" si="10">D17*$B$8/100</f>
         <v>50</v>
       </c>
       <c r="H17" s="1">
-        <f>E17*$B$8/100</f>
+        <f t="shared" si="10"/>
         <v>50</v>
       </c>
       <c r="I17" s="1">
-        <f>F17*$B$8/100</f>
+        <f t="shared" si="10"/>
         <v>50</v>
       </c>
       <c r="J17" s="2"/>
@@ -1236,15 +1271,15 @@
         <v>100</v>
       </c>
       <c r="G18" s="1">
-        <f>D18*$B$8/100</f>
+        <f t="shared" si="10"/>
         <v>50</v>
       </c>
       <c r="H18" s="1">
-        <f>E18*$B$8/100</f>
+        <f t="shared" si="10"/>
         <v>50</v>
       </c>
       <c r="I18" s="1">
-        <f>F18*$B$8/100</f>
+        <f t="shared" si="10"/>
         <v>50</v>
       </c>
       <c r="J18" s="2"/>
@@ -1273,15 +1308,15 @@
         <v>100</v>
       </c>
       <c r="G19" s="1">
-        <f>D19*$B$8/100</f>
+        <f t="shared" si="10"/>
         <v>50</v>
       </c>
       <c r="H19" s="1">
-        <f>E19*$B$8/100</f>
+        <f t="shared" si="10"/>
         <v>50</v>
       </c>
       <c r="I19" s="1">
-        <f>F19*$B$8/100</f>
+        <f t="shared" si="10"/>
         <v>50</v>
       </c>
       <c r="J19" s="2"/>
@@ -2313,10 +2348,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FF0FE83-E5DB-104C-95CA-23FADD2AA11D}">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -2335,7 +2370,7 @@
       <c r="H1" s="5"/>
       <c r="I1" s="5"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -2364,7 +2399,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1">
@@ -2389,7 +2424,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1">
@@ -2414,7 +2449,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
       <c r="B5" s="1">
         <v>90</v>
@@ -2441,7 +2476,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1">
@@ -2466,7 +2501,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1">
@@ -2491,7 +2526,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
       <c r="B8" s="1">
         <v>50</v>
@@ -2500,75 +2535,117 @@
         <v>1</v>
       </c>
       <c r="D8">
+        <v>216</v>
+      </c>
+      <c r="E8" s="1">
+        <v>203</v>
+      </c>
+      <c r="F8" s="1">
+        <v>232</v>
+      </c>
+      <c r="G8">
+        <f>J8/2</f>
+        <v>13</v>
+      </c>
+      <c r="H8">
+        <f t="shared" ref="H8:I8" si="0">K8/2</f>
+        <v>4</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="J8" s="1">
+        <v>26</v>
+      </c>
+      <c r="K8" s="1">
+        <v>8</v>
+      </c>
+      <c r="L8" s="1">
         <v>6</v>
       </c>
-      <c r="E8" s="1">
-        <v>6</v>
-      </c>
-      <c r="F8" s="1">
-        <v>4</v>
-      </c>
-      <c r="G8" s="1">
-        <v>1</v>
-      </c>
-      <c r="H8" s="1">
-        <v>3</v>
-      </c>
-      <c r="I8" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="M8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1">
         <v>2</v>
       </c>
       <c r="D9">
-        <v>4</v>
+        <v>232</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>209</v>
       </c>
       <c r="F9" s="1">
-        <v>4</v>
-      </c>
-      <c r="G9" s="1">
-        <v>0</v>
-      </c>
-      <c r="H9" s="1">
-        <v>0</v>
-      </c>
-      <c r="I9" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+        <v>225</v>
+      </c>
+      <c r="G9">
+        <f t="shared" ref="G9:G10" si="1">J9/2</f>
+        <v>13.5</v>
+      </c>
+      <c r="H9">
+        <f t="shared" ref="H9:H10" si="2">K9/2</f>
+        <v>6.5</v>
+      </c>
+      <c r="I9">
+        <f t="shared" ref="I9:I10" si="3">L9/2</f>
+        <v>4.5</v>
+      </c>
+      <c r="J9" s="1">
+        <v>27</v>
+      </c>
+      <c r="K9" s="1">
+        <v>13</v>
+      </c>
+      <c r="L9" s="1">
+        <v>9</v>
+      </c>
+      <c r="M9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1">
         <v>3</v>
       </c>
       <c r="D10">
-        <v>2</v>
+        <v>125</v>
       </c>
       <c r="E10">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="F10" s="1">
-        <v>3</v>
-      </c>
-      <c r="G10" s="1">
-        <v>0</v>
-      </c>
-      <c r="H10" s="1">
-        <v>0</v>
-      </c>
-      <c r="I10" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+        <v>122</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="1"/>
+        <v>6.5</v>
+      </c>
+      <c r="H10">
+        <f t="shared" si="2"/>
+        <v>3.5</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="3"/>
+        <v>2.5</v>
+      </c>
+      <c r="J10" s="1">
+        <v>13</v>
+      </c>
+      <c r="K10" s="1">
+        <v>7</v>
+      </c>
+      <c r="L10" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>5</v>
       </c>
@@ -2597,7 +2674,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1">
@@ -2622,7 +2699,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1">
@@ -2647,7 +2724,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
       <c r="B14" s="1">
         <v>90</v>
@@ -2674,7 +2751,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1">
@@ -2699,7 +2776,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1">
@@ -2724,7 +2801,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="B17" s="1">
         <v>50</v>
@@ -2750,55 +2827,85 @@
       <c r="I17" s="1">
         <v>9</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="M17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1">
         <v>2</v>
       </c>
       <c r="D18" s="1">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="E18" s="1">
-        <v>1</v>
+        <v>53</v>
       </c>
       <c r="F18" s="1">
-        <v>3</v>
+        <v>41</v>
       </c>
       <c r="G18" s="1">
-        <v>0</v>
+        <f>J18/2</f>
+        <v>14</v>
       </c>
       <c r="H18" s="1">
-        <v>0</v>
+        <f t="shared" ref="H18:I18" si="4">K18/2</f>
+        <v>15</v>
       </c>
       <c r="I18" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+        <f t="shared" si="4"/>
+        <v>11</v>
+      </c>
+      <c r="J18">
+        <v>28</v>
+      </c>
+      <c r="K18">
+        <v>30</v>
+      </c>
+      <c r="L18">
+        <v>22</v>
+      </c>
+      <c r="M18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1">
         <v>3</v>
       </c>
       <c r="D19" s="1">
-        <v>6</v>
+        <v>104</v>
       </c>
       <c r="E19" s="1">
-        <v>4</v>
+        <v>97</v>
       </c>
       <c r="F19" s="1">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="G19" s="1">
-        <v>2</v>
+        <f>J19/2</f>
+        <v>19.5</v>
       </c>
       <c r="H19" s="1">
-        <v>1</v>
+        <f t="shared" ref="H19" si="5">K19/2</f>
+        <v>30</v>
       </c>
       <c r="I19" s="1">
-        <v>1</v>
+        <f t="shared" ref="I19" si="6">L19/2</f>
+        <v>26.5</v>
+      </c>
+      <c r="J19">
+        <v>39</v>
+      </c>
+      <c r="K19">
+        <v>60</v>
+      </c>
+      <c r="L19">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -2808,4 +2915,1338 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0D5EA90-8AEC-854E-B156-1187DEAF50BB}">
+  <dimension ref="A1:M19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1">
+        <v>100</v>
+      </c>
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>63</v>
+      </c>
+      <c r="E2" s="1">
+        <v>53</v>
+      </c>
+      <c r="F2" s="1">
+        <v>72</v>
+      </c>
+      <c r="G2" s="1">
+        <v>69</v>
+      </c>
+      <c r="H2" s="1">
+        <v>59</v>
+      </c>
+      <c r="I2" s="1">
+        <v>53</v>
+      </c>
+      <c r="M2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>75</v>
+      </c>
+      <c r="E3">
+        <v>70</v>
+      </c>
+      <c r="F3" s="1">
+        <v>64</v>
+      </c>
+      <c r="G3" s="1">
+        <v>78</v>
+      </c>
+      <c r="H3" s="1">
+        <v>62</v>
+      </c>
+      <c r="I3" s="1">
+        <v>64</v>
+      </c>
+      <c r="M3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>57</v>
+      </c>
+      <c r="E4">
+        <v>70</v>
+      </c>
+      <c r="F4" s="1">
+        <v>67</v>
+      </c>
+      <c r="G4" s="1">
+        <v>42</v>
+      </c>
+      <c r="H4" s="1">
+        <v>49</v>
+      </c>
+      <c r="I4" s="1">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1">
+        <v>90</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>53</v>
+      </c>
+      <c r="E5" s="1">
+        <v>48</v>
+      </c>
+      <c r="F5" s="1">
+        <v>42</v>
+      </c>
+      <c r="G5">
+        <f>J5/5</f>
+        <v>3.2</v>
+      </c>
+      <c r="H5">
+        <f t="shared" ref="H5:I5" si="0">K5/5</f>
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="0"/>
+        <v>4.2</v>
+      </c>
+      <c r="J5" s="1">
+        <v>16</v>
+      </c>
+      <c r="K5" s="1">
+        <v>11</v>
+      </c>
+      <c r="L5" s="1">
+        <v>21</v>
+      </c>
+      <c r="M5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>55</v>
+      </c>
+      <c r="E6">
+        <v>68</v>
+      </c>
+      <c r="F6" s="1">
+        <v>52</v>
+      </c>
+      <c r="G6">
+        <f t="shared" ref="G6:G7" si="1">J6/5</f>
+        <v>4.8</v>
+      </c>
+      <c r="H6">
+        <f t="shared" ref="H6:H7" si="2">K6/5</f>
+        <v>6.8</v>
+      </c>
+      <c r="I6">
+        <f t="shared" ref="I6:I7" si="3">L6/5</f>
+        <v>5.2</v>
+      </c>
+      <c r="J6" s="1">
+        <v>24</v>
+      </c>
+      <c r="K6" s="1">
+        <v>34</v>
+      </c>
+      <c r="L6" s="1">
+        <v>26</v>
+      </c>
+      <c r="M6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1">
+        <v>3</v>
+      </c>
+      <c r="D7">
+        <v>53</v>
+      </c>
+      <c r="E7">
+        <v>54</v>
+      </c>
+      <c r="F7" s="1">
+        <v>49</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="2"/>
+        <v>5.6</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="3"/>
+        <v>3.6</v>
+      </c>
+      <c r="J7" s="1">
+        <v>20</v>
+      </c>
+      <c r="K7" s="1">
+        <v>28</v>
+      </c>
+      <c r="L7" s="1">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1">
+        <v>50</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>39</v>
+      </c>
+      <c r="E8" s="1">
+        <v>34</v>
+      </c>
+      <c r="F8" s="1">
+        <v>41</v>
+      </c>
+      <c r="G8" s="1">
+        <f>J8/10</f>
+        <v>3</v>
+      </c>
+      <c r="H8" s="1">
+        <f t="shared" ref="H8:I8" si="4">K8/10</f>
+        <v>2.6</v>
+      </c>
+      <c r="I8" s="1">
+        <f t="shared" si="4"/>
+        <v>3.4</v>
+      </c>
+      <c r="J8" s="1">
+        <v>30</v>
+      </c>
+      <c r="K8" s="1">
+        <v>26</v>
+      </c>
+      <c r="L8" s="1">
+        <v>34</v>
+      </c>
+      <c r="M8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1">
+        <v>2</v>
+      </c>
+      <c r="D9">
+        <v>41</v>
+      </c>
+      <c r="E9">
+        <v>41</v>
+      </c>
+      <c r="F9" s="1">
+        <v>32</v>
+      </c>
+      <c r="G9" s="1">
+        <f t="shared" ref="G9:G10" si="5">J9/10</f>
+        <v>4.2</v>
+      </c>
+      <c r="H9" s="1">
+        <f t="shared" ref="H9:H10" si="6">K9/10</f>
+        <v>3.7</v>
+      </c>
+      <c r="I9" s="1">
+        <f t="shared" ref="I9:I10" si="7">L9/10</f>
+        <v>3.1</v>
+      </c>
+      <c r="J9" s="1">
+        <v>42</v>
+      </c>
+      <c r="K9" s="1">
+        <v>37</v>
+      </c>
+      <c r="L9" s="1">
+        <v>31</v>
+      </c>
+      <c r="M9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1">
+        <v>3</v>
+      </c>
+      <c r="D10">
+        <v>39</v>
+      </c>
+      <c r="E10">
+        <v>22</v>
+      </c>
+      <c r="F10" s="1">
+        <v>34</v>
+      </c>
+      <c r="G10" s="1">
+        <f t="shared" si="5"/>
+        <v>3.4</v>
+      </c>
+      <c r="H10" s="1">
+        <f t="shared" si="6"/>
+        <v>3.6</v>
+      </c>
+      <c r="I10" s="1">
+        <f t="shared" si="7"/>
+        <v>1.8</v>
+      </c>
+      <c r="J10" s="1">
+        <v>34</v>
+      </c>
+      <c r="K10" s="1">
+        <v>36</v>
+      </c>
+      <c r="L10" s="1">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="1">
+        <v>100</v>
+      </c>
+      <c r="C11" s="1">
+        <v>1</v>
+      </c>
+      <c r="D11" s="1">
+        <v>32</v>
+      </c>
+      <c r="E11" s="1">
+        <v>34</v>
+      </c>
+      <c r="F11" s="1">
+        <v>41</v>
+      </c>
+      <c r="G11" s="1">
+        <v>34</v>
+      </c>
+      <c r="H11" s="1">
+        <v>35</v>
+      </c>
+      <c r="I11" s="1">
+        <v>27</v>
+      </c>
+      <c r="M11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1">
+        <v>2</v>
+      </c>
+      <c r="D12" s="1">
+        <v>58</v>
+      </c>
+      <c r="E12" s="1">
+        <v>45</v>
+      </c>
+      <c r="F12" s="1">
+        <v>50</v>
+      </c>
+      <c r="G12" s="1">
+        <v>52</v>
+      </c>
+      <c r="H12" s="1">
+        <v>46</v>
+      </c>
+      <c r="I12" s="1">
+        <v>38</v>
+      </c>
+      <c r="M12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1">
+        <v>3</v>
+      </c>
+      <c r="D13" s="1">
+        <v>23</v>
+      </c>
+      <c r="E13" s="1">
+        <v>22</v>
+      </c>
+      <c r="F13" s="1">
+        <v>21</v>
+      </c>
+      <c r="G13" s="1">
+        <v>20</v>
+      </c>
+      <c r="H13" s="1">
+        <v>19</v>
+      </c>
+      <c r="I13" s="1">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1">
+        <v>90</v>
+      </c>
+      <c r="C14" s="1">
+        <v>1</v>
+      </c>
+      <c r="D14" s="1">
+        <v>14</v>
+      </c>
+      <c r="E14" s="1">
+        <v>15</v>
+      </c>
+      <c r="F14" s="1">
+        <v>21</v>
+      </c>
+      <c r="G14" s="1">
+        <v>28</v>
+      </c>
+      <c r="H14" s="1">
+        <v>17</v>
+      </c>
+      <c r="I14" s="1">
+        <v>15</v>
+      </c>
+      <c r="M14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1">
+        <v>2</v>
+      </c>
+      <c r="D15" s="1">
+        <v>29</v>
+      </c>
+      <c r="E15" s="1">
+        <v>21</v>
+      </c>
+      <c r="F15" s="1">
+        <v>37</v>
+      </c>
+      <c r="G15" s="1">
+        <v>32</v>
+      </c>
+      <c r="H15" s="1">
+        <v>17</v>
+      </c>
+      <c r="I15" s="1">
+        <v>18</v>
+      </c>
+      <c r="M15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1">
+        <v>3</v>
+      </c>
+      <c r="D16" s="1">
+        <v>37</v>
+      </c>
+      <c r="E16" s="1">
+        <v>51</v>
+      </c>
+      <c r="F16" s="1">
+        <v>42</v>
+      </c>
+      <c r="G16" s="1">
+        <v>25</v>
+      </c>
+      <c r="H16" s="1">
+        <v>32</v>
+      </c>
+      <c r="I16" s="1">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1">
+        <v>50</v>
+      </c>
+      <c r="C17" s="1">
+        <v>1</v>
+      </c>
+      <c r="D17" s="1">
+        <v>32</v>
+      </c>
+      <c r="E17" s="1">
+        <v>32</v>
+      </c>
+      <c r="F17" s="1">
+        <v>30</v>
+      </c>
+      <c r="G17">
+        <f>J17/10</f>
+        <v>0.8</v>
+      </c>
+      <c r="H17">
+        <f t="shared" ref="H17:I17" si="8">K17/10</f>
+        <v>1.5</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="8"/>
+        <v>1.2</v>
+      </c>
+      <c r="J17" s="1">
+        <v>8</v>
+      </c>
+      <c r="K17" s="1">
+        <v>15</v>
+      </c>
+      <c r="L17" s="1">
+        <v>12</v>
+      </c>
+      <c r="M17" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1">
+        <v>2</v>
+      </c>
+      <c r="D18" s="1">
+        <v>39</v>
+      </c>
+      <c r="E18" s="1">
+        <v>39</v>
+      </c>
+      <c r="F18" s="1">
+        <v>32</v>
+      </c>
+      <c r="G18">
+        <f t="shared" ref="G18:G19" si="9">J18/10</f>
+        <v>0.7</v>
+      </c>
+      <c r="H18">
+        <f t="shared" ref="H18:H19" si="10">K18/10</f>
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="I18">
+        <f t="shared" ref="I18:I19" si="11">L18/10</f>
+        <v>1.2</v>
+      </c>
+      <c r="J18" s="1">
+        <v>7</v>
+      </c>
+      <c r="K18" s="1">
+        <v>11</v>
+      </c>
+      <c r="L18" s="1">
+        <v>12</v>
+      </c>
+      <c r="M18" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1">
+        <v>3</v>
+      </c>
+      <c r="D19" s="1">
+        <v>11</v>
+      </c>
+      <c r="E19" s="1">
+        <v>17</v>
+      </c>
+      <c r="F19" s="1">
+        <v>11</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="9"/>
+        <v>0.6</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="10"/>
+        <v>0.4</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="11"/>
+        <v>0.9</v>
+      </c>
+      <c r="J19" s="1">
+        <v>6</v>
+      </c>
+      <c r="K19" s="1">
+        <v>4</v>
+      </c>
+      <c r="L19" s="1">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="J1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CD2B6D8-38EE-8F44-B9AE-A92FB72BA086}">
+  <dimension ref="A1:M19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1">
+        <v>100</v>
+      </c>
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>77</v>
+      </c>
+      <c r="E2" s="1">
+        <v>84</v>
+      </c>
+      <c r="F2" s="1">
+        <v>94</v>
+      </c>
+      <c r="G2" s="1">
+        <v>27</v>
+      </c>
+      <c r="H2" s="1">
+        <v>38</v>
+      </c>
+      <c r="I2" s="1"/>
+      <c r="M2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>77</v>
+      </c>
+      <c r="E3">
+        <v>100</v>
+      </c>
+      <c r="F3" s="1">
+        <v>120</v>
+      </c>
+      <c r="G3" s="1">
+        <v>31</v>
+      </c>
+      <c r="H3" s="1">
+        <v>40</v>
+      </c>
+      <c r="I3" s="1"/>
+      <c r="M3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>56</v>
+      </c>
+      <c r="E4">
+        <v>53</v>
+      </c>
+      <c r="F4" s="1">
+        <v>72</v>
+      </c>
+      <c r="G4" s="1">
+        <v>13</v>
+      </c>
+      <c r="H4" s="1">
+        <v>20</v>
+      </c>
+      <c r="I4" s="1"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1">
+        <v>90</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>84</v>
+      </c>
+      <c r="E5" s="1">
+        <v>96</v>
+      </c>
+      <c r="F5" s="1">
+        <v>88</v>
+      </c>
+      <c r="G5">
+        <f>J5/20</f>
+        <v>4.5</v>
+      </c>
+      <c r="H5">
+        <f t="shared" ref="H5:I5" si="0">K5/20</f>
+        <v>5.4</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="0"/>
+        <v>4.6500000000000004</v>
+      </c>
+      <c r="J5">
+        <v>90</v>
+      </c>
+      <c r="K5" s="1">
+        <v>108</v>
+      </c>
+      <c r="L5" s="1">
+        <v>93</v>
+      </c>
+      <c r="M5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>26</v>
+      </c>
+      <c r="E6">
+        <v>26</v>
+      </c>
+      <c r="F6" s="1">
+        <v>27</v>
+      </c>
+      <c r="G6">
+        <f t="shared" ref="G6:G7" si="1">J6/20</f>
+        <v>2.5</v>
+      </c>
+      <c r="H6">
+        <f t="shared" ref="H6:H7" si="2">K6/20</f>
+        <v>3.1</v>
+      </c>
+      <c r="I6">
+        <f t="shared" ref="I6:I7" si="3">L6/20</f>
+        <v>2.1</v>
+      </c>
+      <c r="J6" s="1">
+        <v>50</v>
+      </c>
+      <c r="K6" s="1">
+        <v>62</v>
+      </c>
+      <c r="L6" s="1">
+        <v>42</v>
+      </c>
+      <c r="M6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1">
+        <v>3</v>
+      </c>
+      <c r="D7">
+        <v>8</v>
+      </c>
+      <c r="E7">
+        <v>9</v>
+      </c>
+      <c r="F7" s="1">
+        <v>8</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="1"/>
+        <v>0.35</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="2"/>
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="3"/>
+        <v>0.45</v>
+      </c>
+      <c r="J7" s="1">
+        <v>7</v>
+      </c>
+      <c r="K7" s="1">
+        <v>11</v>
+      </c>
+      <c r="L7" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1">
+        <v>50</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>44</v>
+      </c>
+      <c r="E8" s="1">
+        <v>42</v>
+      </c>
+      <c r="F8" s="1">
+        <v>39</v>
+      </c>
+      <c r="G8" s="1">
+        <f>J8/10</f>
+        <v>2.6</v>
+      </c>
+      <c r="H8" s="1">
+        <f t="shared" ref="H8" si="4">K8/10</f>
+        <v>3</v>
+      </c>
+      <c r="I8" s="1">
+        <f t="shared" ref="I8" si="5">L8/10</f>
+        <v>2.9</v>
+      </c>
+      <c r="J8" s="1">
+        <v>26</v>
+      </c>
+      <c r="K8" s="1">
+        <v>30</v>
+      </c>
+      <c r="L8" s="1">
+        <v>29</v>
+      </c>
+      <c r="M8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1">
+        <v>2</v>
+      </c>
+      <c r="D9">
+        <v>32</v>
+      </c>
+      <c r="E9">
+        <v>41</v>
+      </c>
+      <c r="F9" s="1">
+        <v>39</v>
+      </c>
+      <c r="G9" s="1">
+        <f t="shared" ref="G9:G10" si="6">J9/10</f>
+        <v>3.8</v>
+      </c>
+      <c r="H9" s="1">
+        <f t="shared" ref="H9:H10" si="7">K9/10</f>
+        <v>3.8</v>
+      </c>
+      <c r="I9" s="1">
+        <f t="shared" ref="I9:I10" si="8">L9/10</f>
+        <v>3.4</v>
+      </c>
+      <c r="J9" s="1">
+        <v>38</v>
+      </c>
+      <c r="K9" s="1">
+        <v>38</v>
+      </c>
+      <c r="L9" s="1">
+        <v>34</v>
+      </c>
+      <c r="M9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1">
+        <v>3</v>
+      </c>
+      <c r="D10">
+        <v>42</v>
+      </c>
+      <c r="E10">
+        <v>51</v>
+      </c>
+      <c r="F10" s="1">
+        <v>48</v>
+      </c>
+      <c r="G10" s="1">
+        <f t="shared" si="6"/>
+        <v>3.1</v>
+      </c>
+      <c r="H10" s="1">
+        <f t="shared" si="7"/>
+        <v>3.2</v>
+      </c>
+      <c r="I10" s="1">
+        <f t="shared" si="8"/>
+        <v>3.3</v>
+      </c>
+      <c r="J10" s="1">
+        <v>31</v>
+      </c>
+      <c r="K10" s="1">
+        <v>32</v>
+      </c>
+      <c r="L10" s="1">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="1">
+        <v>100</v>
+      </c>
+      <c r="C11" s="1">
+        <v>1</v>
+      </c>
+      <c r="D11" s="1">
+        <v>72</v>
+      </c>
+      <c r="E11" s="1">
+        <v>86</v>
+      </c>
+      <c r="F11" s="1">
+        <v>56</v>
+      </c>
+      <c r="G11" s="1">
+        <v>74</v>
+      </c>
+      <c r="H11" s="1">
+        <v>76</v>
+      </c>
+      <c r="I11" s="1">
+        <v>54</v>
+      </c>
+      <c r="M11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1">
+        <v>2</v>
+      </c>
+      <c r="D12" s="1">
+        <v>76</v>
+      </c>
+      <c r="E12" s="1">
+        <v>95</v>
+      </c>
+      <c r="F12" s="1">
+        <v>68</v>
+      </c>
+      <c r="G12" s="1">
+        <v>80</v>
+      </c>
+      <c r="H12" s="1">
+        <v>60</v>
+      </c>
+      <c r="I12" s="1">
+        <v>65</v>
+      </c>
+      <c r="M12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1">
+        <v>3</v>
+      </c>
+      <c r="D13" s="1">
+        <v>31</v>
+      </c>
+      <c r="E13" s="1">
+        <v>30</v>
+      </c>
+      <c r="F13" s="1">
+        <v>40</v>
+      </c>
+      <c r="G13" s="1">
+        <v>36</v>
+      </c>
+      <c r="H13" s="1">
+        <v>37</v>
+      </c>
+      <c r="I13" s="1">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1">
+        <v>90</v>
+      </c>
+      <c r="C14" s="1">
+        <v>1</v>
+      </c>
+      <c r="D14" s="1">
+        <v>21</v>
+      </c>
+      <c r="E14" s="1">
+        <v>27</v>
+      </c>
+      <c r="F14" s="1">
+        <v>27</v>
+      </c>
+      <c r="G14" s="1">
+        <f>J14/5</f>
+        <v>17</v>
+      </c>
+      <c r="H14" s="1">
+        <f t="shared" ref="H14:I14" si="9">K14/5</f>
+        <v>14.6</v>
+      </c>
+      <c r="I14" s="1">
+        <f t="shared" si="9"/>
+        <v>11.6</v>
+      </c>
+      <c r="J14">
+        <v>85</v>
+      </c>
+      <c r="K14">
+        <v>73</v>
+      </c>
+      <c r="L14">
+        <v>58</v>
+      </c>
+      <c r="M14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1">
+        <v>2</v>
+      </c>
+      <c r="D15" s="1">
+        <v>15</v>
+      </c>
+      <c r="E15" s="1">
+        <v>18</v>
+      </c>
+      <c r="F15" s="1">
+        <v>19</v>
+      </c>
+      <c r="G15" s="1">
+        <f t="shared" ref="G15:G16" si="10">J15/5</f>
+        <v>11.8</v>
+      </c>
+      <c r="H15" s="1">
+        <f t="shared" ref="H15:H16" si="11">K15/5</f>
+        <v>9.6</v>
+      </c>
+      <c r="I15" s="1">
+        <f t="shared" ref="I15:I16" si="12">L15/5</f>
+        <v>8</v>
+      </c>
+      <c r="J15">
+        <v>59</v>
+      </c>
+      <c r="K15">
+        <v>48</v>
+      </c>
+      <c r="L15">
+        <v>40</v>
+      </c>
+      <c r="M15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1">
+        <v>3</v>
+      </c>
+      <c r="D16" s="1">
+        <v>26</v>
+      </c>
+      <c r="E16" s="1">
+        <v>25</v>
+      </c>
+      <c r="F16" s="1">
+        <v>30</v>
+      </c>
+      <c r="G16" s="1">
+        <f t="shared" si="10"/>
+        <v>13</v>
+      </c>
+      <c r="H16" s="1">
+        <f t="shared" si="11"/>
+        <v>14</v>
+      </c>
+      <c r="I16" s="1">
+        <f t="shared" si="12"/>
+        <v>15.8</v>
+      </c>
+      <c r="J16">
+        <v>65</v>
+      </c>
+      <c r="K16">
+        <v>70</v>
+      </c>
+      <c r="L16">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1">
+        <v>50</v>
+      </c>
+      <c r="C17" s="1">
+        <v>1</v>
+      </c>
+      <c r="D17" s="1">
+        <v>51</v>
+      </c>
+      <c r="E17" s="1">
+        <v>49</v>
+      </c>
+      <c r="F17" s="1">
+        <v>49</v>
+      </c>
+      <c r="G17">
+        <f>J17/10</f>
+        <v>7.1</v>
+      </c>
+      <c r="H17">
+        <f t="shared" ref="H17:I17" si="13">K17/10</f>
+        <v>6.9</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="13"/>
+        <v>5.5</v>
+      </c>
+      <c r="J17" s="1">
+        <v>71</v>
+      </c>
+      <c r="K17" s="1">
+        <v>69</v>
+      </c>
+      <c r="L17" s="1">
+        <v>55</v>
+      </c>
+      <c r="M17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1">
+        <v>2</v>
+      </c>
+      <c r="D18" s="1">
+        <v>40</v>
+      </c>
+      <c r="E18" s="1">
+        <v>47</v>
+      </c>
+      <c r="F18" s="1">
+        <v>52</v>
+      </c>
+      <c r="G18">
+        <f t="shared" ref="G18:G19" si="14">J18/10</f>
+        <v>5.7</v>
+      </c>
+      <c r="H18">
+        <f t="shared" ref="H18:H19" si="15">K18/10</f>
+        <v>4.7</v>
+      </c>
+      <c r="I18">
+        <f t="shared" ref="I18:I19" si="16">L18/10</f>
+        <v>5</v>
+      </c>
+      <c r="J18" s="1">
+        <v>57</v>
+      </c>
+      <c r="K18" s="1">
+        <v>47</v>
+      </c>
+      <c r="L18" s="1">
+        <v>50</v>
+      </c>
+      <c r="M18" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1">
+        <v>3</v>
+      </c>
+      <c r="D19" s="1">
+        <v>29</v>
+      </c>
+      <c r="E19" s="1">
+        <v>37</v>
+      </c>
+      <c r="F19" s="1">
+        <v>36</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="14"/>
+        <v>3.8</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="15"/>
+        <v>4.2</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="16"/>
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="J19" s="1">
+        <v>38</v>
+      </c>
+      <c r="K19" s="1">
+        <v>42</v>
+      </c>
+      <c r="L19" s="1">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="J1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>